<commit_message>
add cheering dyad partners to cow-herding minigame
</commit_message>
<xml_diff>
--- a/tools/game_levels.xlsx
+++ b/tools/game_levels.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/severin/Uni/Work/pydew-valley-uzh-dyadic/tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{819C46D7-6EEE-4B40-A94A-30535F8D52B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF95CC3-82D0-9C4D-9728-5239131187BE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="51200" windowHeight="28300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,12 +17,25 @@
     <sheet name="v2 (friend version)" sheetId="2" r:id="rId2"/>
     <sheet name="v3 (no group version)" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="247">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="246">
   <si>
     <t>Feature</t>
   </si>
@@ -739,9 +752,6 @@
   </si>
   <si>
     <t>15min</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No </t>
   </si>
   <si>
     <t>clan_intro_solo</t>
@@ -781,31 +791,37 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1033,8 +1049,8 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1050,8 +1066,8 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2392,7 +2408,7 @@
       <c r="M39" s="25"/>
       <c r="N39" s="26"/>
     </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A40" s="11" t="s">
         <v>153</v>
       </c>
@@ -2436,14 +2452,14 @@
         <v>0.62152777777777779</v>
       </c>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
         <v>155</v>
       </c>
       <c r="B41" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="C41" s="27" t="s">
+      <c r="C41" s="34" t="s">
         <v>20</v>
       </c>
       <c r="D41" s="25"/>
@@ -2451,7 +2467,7 @@
       <c r="F41" s="25"/>
       <c r="G41" s="25"/>
       <c r="H41" s="26"/>
-      <c r="I41" s="27" t="s">
+      <c r="I41" s="34" t="s">
         <v>20</v>
       </c>
       <c r="J41" s="25"/>
@@ -6886,44 +6902,15 @@
     </row>
   </sheetData>
   <mergeCells count="64">
-    <mergeCell ref="I47:N47"/>
-    <mergeCell ref="I67:N67"/>
-    <mergeCell ref="I68:N68"/>
-    <mergeCell ref="C67:H67"/>
-    <mergeCell ref="C68:H68"/>
-    <mergeCell ref="C47:H47"/>
-    <mergeCell ref="C65:H65"/>
-    <mergeCell ref="C66:H66"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C39:H39"/>
-    <mergeCell ref="I43:N43"/>
-    <mergeCell ref="J45:N45"/>
-    <mergeCell ref="I46:N46"/>
-    <mergeCell ref="C41:H41"/>
-    <mergeCell ref="C43:H43"/>
-    <mergeCell ref="C45:H45"/>
-    <mergeCell ref="C46:H46"/>
-    <mergeCell ref="C27:H27"/>
-    <mergeCell ref="C28:H28"/>
-    <mergeCell ref="C29:H29"/>
-    <mergeCell ref="C30:H30"/>
-    <mergeCell ref="C31:H31"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
-    <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C26:H26"/>
-    <mergeCell ref="C19:H19"/>
-    <mergeCell ref="I19:N19"/>
-    <mergeCell ref="J20:N20"/>
-    <mergeCell ref="C20:H20"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="I9:N9"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="I10:N10"/>
-    <mergeCell ref="C17:H17"/>
-    <mergeCell ref="I17:N17"/>
+    <mergeCell ref="J22:N22"/>
+    <mergeCell ref="J23:N23"/>
+    <mergeCell ref="I24:N24"/>
+    <mergeCell ref="I25:N25"/>
+    <mergeCell ref="I26:N26"/>
+    <mergeCell ref="I27:N27"/>
+    <mergeCell ref="I28:N28"/>
+    <mergeCell ref="I29:N29"/>
+    <mergeCell ref="I30:N30"/>
     <mergeCell ref="I31:N31"/>
     <mergeCell ref="I32:N32"/>
     <mergeCell ref="I39:N39"/>
@@ -6940,16 +6927,45 @@
     <mergeCell ref="I7:N7"/>
     <mergeCell ref="C8:H8"/>
     <mergeCell ref="I8:N8"/>
-    <mergeCell ref="I26:N26"/>
-    <mergeCell ref="I27:N27"/>
-    <mergeCell ref="I28:N28"/>
-    <mergeCell ref="I29:N29"/>
-    <mergeCell ref="I30:N30"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="I9:N9"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="I10:N10"/>
+    <mergeCell ref="C17:H17"/>
+    <mergeCell ref="I17:N17"/>
+    <mergeCell ref="C19:H19"/>
+    <mergeCell ref="I19:N19"/>
+    <mergeCell ref="J20:N20"/>
+    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C21:H21"/>
     <mergeCell ref="J21:N21"/>
-    <mergeCell ref="J22:N22"/>
-    <mergeCell ref="J23:N23"/>
-    <mergeCell ref="I24:N24"/>
-    <mergeCell ref="I25:N25"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="C28:H28"/>
+    <mergeCell ref="C29:H29"/>
+    <mergeCell ref="C30:H30"/>
+    <mergeCell ref="C31:H31"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C39:H39"/>
+    <mergeCell ref="I43:N43"/>
+    <mergeCell ref="J45:N45"/>
+    <mergeCell ref="I46:N46"/>
+    <mergeCell ref="C41:H41"/>
+    <mergeCell ref="C43:H43"/>
+    <mergeCell ref="C45:H45"/>
+    <mergeCell ref="C46:H46"/>
+    <mergeCell ref="I47:N47"/>
+    <mergeCell ref="I67:N67"/>
+    <mergeCell ref="I68:N68"/>
+    <mergeCell ref="C67:H67"/>
+    <mergeCell ref="C68:H68"/>
+    <mergeCell ref="C47:H47"/>
+    <mergeCell ref="C65:H65"/>
+    <mergeCell ref="C66:H66"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -8093,7 +8109,7 @@
       <c r="M40" s="25"/>
       <c r="N40" s="26"/>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
         <v>153</v>
       </c>
@@ -8137,14 +8153,14 @@
         <v>0.62152777777777779</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
         <v>155</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="C42" s="27" t="s">
+      <c r="C42" s="34" t="s">
         <v>20</v>
       </c>
       <c r="D42" s="25"/>
@@ -8152,7 +8168,7 @@
       <c r="F42" s="25"/>
       <c r="G42" s="25"/>
       <c r="H42" s="26"/>
-      <c r="I42" s="27" t="s">
+      <c r="I42" s="34" t="s">
         <v>20</v>
       </c>
       <c r="J42" s="25"/>
@@ -12587,6 +12603,58 @@
     </row>
   </sheetData>
   <mergeCells count="66">
+    <mergeCell ref="J21:N21"/>
+    <mergeCell ref="J22:N22"/>
+    <mergeCell ref="J23:N23"/>
+    <mergeCell ref="I25:N25"/>
+    <mergeCell ref="I26:N26"/>
+    <mergeCell ref="I27:N27"/>
+    <mergeCell ref="I28:N28"/>
+    <mergeCell ref="I29:N29"/>
+    <mergeCell ref="I30:N30"/>
+    <mergeCell ref="I31:N31"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="I5:N5"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="I6:N6"/>
+    <mergeCell ref="C7:H7"/>
+    <mergeCell ref="I7:N7"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:N1"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="I4:N4"/>
+    <mergeCell ref="I8:N8"/>
+    <mergeCell ref="I9:N9"/>
+    <mergeCell ref="I10:N10"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="C17:H17"/>
+    <mergeCell ref="I17:N17"/>
+    <mergeCell ref="C19:H19"/>
+    <mergeCell ref="I19:N19"/>
+    <mergeCell ref="J20:N20"/>
+    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="C28:H28"/>
+    <mergeCell ref="C29:H29"/>
+    <mergeCell ref="C30:H30"/>
+    <mergeCell ref="C31:H31"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="I44:N44"/>
+    <mergeCell ref="J46:N46"/>
+    <mergeCell ref="I32:N32"/>
+    <mergeCell ref="I33:N33"/>
+    <mergeCell ref="I40:N40"/>
+    <mergeCell ref="I42:N42"/>
     <mergeCell ref="C69:H69"/>
     <mergeCell ref="I69:N69"/>
     <mergeCell ref="C40:H40"/>
@@ -12601,58 +12669,6 @@
     <mergeCell ref="C67:H67"/>
     <mergeCell ref="C68:H68"/>
     <mergeCell ref="I68:N68"/>
-    <mergeCell ref="C31:H31"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="I44:N44"/>
-    <mergeCell ref="J46:N46"/>
-    <mergeCell ref="C26:H26"/>
-    <mergeCell ref="C27:H27"/>
-    <mergeCell ref="C28:H28"/>
-    <mergeCell ref="C29:H29"/>
-    <mergeCell ref="C30:H30"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
-    <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C17:H17"/>
-    <mergeCell ref="I17:N17"/>
-    <mergeCell ref="C19:H19"/>
-    <mergeCell ref="I19:N19"/>
-    <mergeCell ref="J20:N20"/>
-    <mergeCell ref="C20:H20"/>
-    <mergeCell ref="I8:N8"/>
-    <mergeCell ref="I9:N9"/>
-    <mergeCell ref="I10:N10"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="I32:N32"/>
-    <mergeCell ref="I33:N33"/>
-    <mergeCell ref="I40:N40"/>
-    <mergeCell ref="I42:N42"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:N1"/>
-    <mergeCell ref="C4:H4"/>
-    <mergeCell ref="I4:N4"/>
-    <mergeCell ref="C5:H5"/>
-    <mergeCell ref="I5:N5"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="I6:N6"/>
-    <mergeCell ref="C7:H7"/>
-    <mergeCell ref="I7:N7"/>
-    <mergeCell ref="C8:H8"/>
-    <mergeCell ref="I27:N27"/>
-    <mergeCell ref="I28:N28"/>
-    <mergeCell ref="I29:N29"/>
-    <mergeCell ref="I30:N30"/>
-    <mergeCell ref="I31:N31"/>
-    <mergeCell ref="J21:N21"/>
-    <mergeCell ref="J22:N22"/>
-    <mergeCell ref="J23:N23"/>
-    <mergeCell ref="I25:N25"/>
-    <mergeCell ref="I26:N26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -13187,7 +13203,7 @@
       <c r="F19" s="25"/>
       <c r="G19" s="25"/>
       <c r="H19" s="26"/>
-      <c r="I19" s="34" t="s">
+      <c r="I19" s="27" t="s">
         <v>29</v>
       </c>
       <c r="J19" s="25"/>
@@ -13784,7 +13800,7 @@
       <c r="M40" s="22"/>
       <c r="N40" s="23"/>
     </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A41" s="11" t="s">
         <v>153</v>
       </c>
@@ -13828,14 +13844,14 @@
         <v>0.62152777777777779</v>
       </c>
     </row>
-    <row r="42" spans="1:14" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A42" s="11" t="s">
         <v>155</v>
       </c>
       <c r="B42" s="11" t="s">
         <v>156</v>
       </c>
-      <c r="C42" s="27" t="s">
+      <c r="C42" s="34" t="s">
         <v>20</v>
       </c>
       <c r="D42" s="25"/>
@@ -13843,7 +13859,7 @@
       <c r="F42" s="25"/>
       <c r="G42" s="25"/>
       <c r="H42" s="26"/>
-      <c r="I42" s="27" t="s">
+      <c r="I42" s="34" t="s">
         <v>20</v>
       </c>
       <c r="J42" s="25"/>
@@ -13996,7 +14012,7 @@
         <v>169</v>
       </c>
       <c r="C48" s="24" t="s">
-        <v>239</v>
+        <v>20</v>
       </c>
       <c r="D48" s="25"/>
       <c r="E48" s="25"/>
@@ -14018,7 +14034,7 @@
         <v>171</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D49" s="4"/>
       <c r="E49" s="4"/>
@@ -14040,7 +14056,7 @@
         <v>174</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D50" s="7"/>
       <c r="E50" s="4"/>
@@ -14062,7 +14078,7 @@
         <v>177</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D51" s="7"/>
       <c r="E51" s="4"/>
@@ -14078,13 +14094,13 @@
     </row>
     <row r="52" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A52" s="5" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>180</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D52" s="7"/>
       <c r="E52" s="4"/>
@@ -14106,7 +14122,7 @@
         <v>183</v>
       </c>
       <c r="C53" s="9" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D53" s="7"/>
       <c r="E53" s="4"/>
@@ -14272,7 +14288,7 @@
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="F61" s="4"/>
       <c r="G61" s="4"/>
@@ -18222,6 +18238,55 @@
     </row>
   </sheetData>
   <mergeCells count="65">
+    <mergeCell ref="C40:H40"/>
+    <mergeCell ref="C42:H42"/>
+    <mergeCell ref="I42:N42"/>
+    <mergeCell ref="C44:H44"/>
+    <mergeCell ref="I44:N44"/>
+    <mergeCell ref="C46:H46"/>
+    <mergeCell ref="J46:N46"/>
+    <mergeCell ref="C68:H68"/>
+    <mergeCell ref="C69:H69"/>
+    <mergeCell ref="C47:H47"/>
+    <mergeCell ref="I47:N47"/>
+    <mergeCell ref="C48:H48"/>
+    <mergeCell ref="I48:N48"/>
+    <mergeCell ref="C66:H66"/>
+    <mergeCell ref="C67:H67"/>
+    <mergeCell ref="I68:N68"/>
+    <mergeCell ref="I69:N69"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="C1:N1"/>
+    <mergeCell ref="C4:H4"/>
+    <mergeCell ref="I4:N4"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="I5:N5"/>
+    <mergeCell ref="C6:H6"/>
+    <mergeCell ref="I6:N6"/>
+    <mergeCell ref="C7:H7"/>
+    <mergeCell ref="I7:N7"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="I8:N8"/>
+    <mergeCell ref="I9:N9"/>
+    <mergeCell ref="I10:N10"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="C10:H10"/>
+    <mergeCell ref="C17:H17"/>
+    <mergeCell ref="I17:N17"/>
+    <mergeCell ref="C19:H19"/>
+    <mergeCell ref="I19:N19"/>
+    <mergeCell ref="J20:N20"/>
+    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="C29:H29"/>
+    <mergeCell ref="C30:H30"/>
+    <mergeCell ref="C31:H31"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="C21:H21"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="C24:H24"/>
+    <mergeCell ref="C25:H25"/>
     <mergeCell ref="C33:H33"/>
     <mergeCell ref="I33:N33"/>
     <mergeCell ref="J21:N21"/>
@@ -18238,55 +18303,6 @@
     <mergeCell ref="I32:N32"/>
     <mergeCell ref="C27:H27"/>
     <mergeCell ref="C28:H28"/>
-    <mergeCell ref="C29:H29"/>
-    <mergeCell ref="C30:H30"/>
-    <mergeCell ref="C31:H31"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="C21:H21"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="C23:H23"/>
-    <mergeCell ref="C24:H24"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="C17:H17"/>
-    <mergeCell ref="I17:N17"/>
-    <mergeCell ref="C19:H19"/>
-    <mergeCell ref="I19:N19"/>
-    <mergeCell ref="J20:N20"/>
-    <mergeCell ref="C20:H20"/>
-    <mergeCell ref="C8:H8"/>
-    <mergeCell ref="I8:N8"/>
-    <mergeCell ref="I9:N9"/>
-    <mergeCell ref="I10:N10"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="C10:H10"/>
-    <mergeCell ref="C5:H5"/>
-    <mergeCell ref="I5:N5"/>
-    <mergeCell ref="C6:H6"/>
-    <mergeCell ref="I6:N6"/>
-    <mergeCell ref="C7:H7"/>
-    <mergeCell ref="I7:N7"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="C1:N1"/>
-    <mergeCell ref="C4:H4"/>
-    <mergeCell ref="I4:N4"/>
-    <mergeCell ref="C46:H46"/>
-    <mergeCell ref="J46:N46"/>
-    <mergeCell ref="C68:H68"/>
-    <mergeCell ref="C69:H69"/>
-    <mergeCell ref="C47:H47"/>
-    <mergeCell ref="I47:N47"/>
-    <mergeCell ref="C48:H48"/>
-    <mergeCell ref="I48:N48"/>
-    <mergeCell ref="C66:H66"/>
-    <mergeCell ref="C67:H67"/>
-    <mergeCell ref="I68:N68"/>
-    <mergeCell ref="I69:N69"/>
-    <mergeCell ref="C40:H40"/>
-    <mergeCell ref="C42:H42"/>
-    <mergeCell ref="I42:N42"/>
-    <mergeCell ref="C44:H44"/>
-    <mergeCell ref="I44:N44"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>